<commit_message>
new changes added 19/01/2025
</commit_message>
<xml_diff>
--- a/test_file.xlsx
+++ b/test_file.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Divyesh\IFC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Divyesh\IFC\AmazonDB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31435541-8950-4F6C-8AF5-2E894FD2B5A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9D969A1-7C60-4464-BD4F-60F947FFC387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -147,9 +147,6 @@
     <t>DONE</t>
   </si>
   <si>
-    <t>Customer acquisition &amp; credibility check (credit risk analysis)</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Customer </t>
     </r>
@@ -254,9 +251,6 @@
   </si>
   <si>
     <t>Non-financial (Revenue from Operations &amp; Other Income)</t>
-  </si>
-  <si>
-    <t>Sales Order Confirmation &amp; Closing</t>
   </si>
   <si>
     <t>Sales Order Confirmation</t>
@@ -372,6 +366,12 @@
   </si>
   <si>
     <t>divyesh.parmar@sharpandtannan.com</t>
+  </si>
+  <si>
+    <t>Customer Testing (credit risk analysis)</t>
+  </si>
+  <si>
+    <t>Sales Order Testing</t>
   </si>
 </sst>
 </file>
@@ -447,7 +447,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -468,19 +468,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -532,7 +520,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -566,31 +554,19 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -599,7 +575,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
@@ -1044,145 +1020,145 @@
       <c r="AC2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="AD2" s="19" t="s">
+      <c r="AD2" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="AE2" s="22" t="s">
-        <v>74</v>
+      <c r="AE2" s="18" t="s">
+        <v>72</v>
       </c>
       <c r="AF2" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="AG2" s="14" t="s">
+      <c r="AG2" s="12" t="s">
         <v>28</v>
       </c>
       <c r="AH2" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
-    <row r="3" spans="1:34" s="3" customFormat="1" ht="144" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:34" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="6"/>
-      <c r="B3" s="7">
-        <v>1</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="H3" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="I3" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="K3" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="L3" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="M3" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="N3" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="O3" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="P3" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q3" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="R3" s="8" t="s">
-        <v>48</v>
-      </c>
+      <c r="B3" s="7"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="8"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="8"/>
       <c r="S3" s="10"/>
       <c r="T3" s="10"/>
       <c r="U3" s="10"/>
       <c r="V3" s="10"/>
       <c r="W3" s="10"/>
       <c r="X3" s="10"/>
-      <c r="Y3" s="8" t="s">
+      <c r="Y3" s="8"/>
+      <c r="Z3" s="8"/>
+      <c r="AA3" s="8"/>
+      <c r="AB3" s="8"/>
+      <c r="AC3" s="8"/>
+      <c r="AD3" s="8"/>
+      <c r="AF3" s="8"/>
+      <c r="AG3" s="8"/>
+    </row>
+    <row r="4" spans="1:34" s="3" customFormat="1" ht="144" x14ac:dyDescent="0.2">
+      <c r="A4" s="6"/>
+      <c r="B4" s="7">
+        <v>1</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="M4" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="N4" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O4" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="P4" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q4" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="R4" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="S4" s="10"/>
+      <c r="T4" s="10"/>
+      <c r="U4" s="10"/>
+      <c r="V4" s="10"/>
+      <c r="W4" s="10"/>
+      <c r="X4" s="10"/>
+      <c r="Y4" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z4" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA4" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="Z3" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA3" s="8" t="s">
+      <c r="AB4" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="AB3" s="8" t="s">
+      <c r="AC4" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="AC3" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD3" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="AE3" s="3" t="s">
+      <c r="AD4" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="AE4" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="AF4" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="AG4" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="AH4" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="AF3" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="AG3" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="AH3" s="3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="4" spans="1:34" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="6"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="8"/>
-      <c r="L4" s="8"/>
-      <c r="M4" s="8"/>
-      <c r="N4" s="8"/>
-      <c r="O4" s="8"/>
-      <c r="P4" s="8"/>
-      <c r="Q4" s="8"/>
-      <c r="R4" s="8"/>
-      <c r="S4" s="12"/>
-      <c r="T4" s="12"/>
-      <c r="U4" s="12"/>
-      <c r="V4" s="12"/>
-      <c r="W4" s="12"/>
-      <c r="X4" s="12"/>
-      <c r="Y4" s="9"/>
-      <c r="Z4" s="8"/>
-      <c r="AA4" s="8"/>
-      <c r="AB4" s="8"/>
-      <c r="AC4" s="8"/>
-      <c r="AD4" s="8"/>
-      <c r="AF4" s="8"/>
-      <c r="AG4" s="8"/>
     </row>
     <row r="5" spans="1:34" ht="127.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6"/>
@@ -1203,12 +1179,12 @@
       <c r="P5" s="8"/>
       <c r="Q5" s="8"/>
       <c r="R5" s="8"/>
-      <c r="S5" s="13"/>
-      <c r="T5" s="13"/>
-      <c r="U5" s="13"/>
-      <c r="V5" s="13"/>
-      <c r="W5" s="13"/>
-      <c r="X5" s="13"/>
+      <c r="S5" s="11"/>
+      <c r="T5" s="11"/>
+      <c r="U5" s="11"/>
+      <c r="V5" s="11"/>
+      <c r="W5" s="11"/>
+      <c r="X5" s="11"/>
       <c r="Y5" s="8"/>
       <c r="Z5" s="8"/>
       <c r="AA5" s="8"/>
@@ -1222,7 +1198,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="Q3" r:id="rId1" xr:uid="{355510E2-467C-4A91-A76D-5D5C14FF4268}"/>
+    <hyperlink ref="Q4" r:id="rId1" xr:uid="{27249811-1D22-4D47-AA96-D2E1E20EBF9B}"/>
   </hyperlinks>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="50" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId2"/>
@@ -1357,153 +1333,150 @@
       <c r="AD2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="AE2" s="22" t="s">
+      <c r="AE2" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="AF2" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="AG2" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="AH2" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="AF2" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="AG2" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="AH2" s="3" t="s">
-        <v>76</v>
-      </c>
     </row>
-    <row r="3" spans="1:34" s="3" customFormat="1" ht="108" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:34" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="6"/>
-      <c r="B3" s="7">
-        <f>3+1</f>
-        <v>4</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H3" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="I3" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="K3" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="L3" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="M3" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="N3" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="O3" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="P3" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q3" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="R3" s="8" t="s">
-        <v>66</v>
-      </c>
+      <c r="B3" s="7"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="8"/>
+      <c r="P3" s="8"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="8"/>
       <c r="S3" s="10"/>
       <c r="T3" s="10"/>
       <c r="U3" s="10"/>
       <c r="V3" s="10"/>
       <c r="W3" s="10"/>
       <c r="X3" s="10"/>
-      <c r="Y3" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="Z3" s="8" t="s">
+      <c r="Y3" s="8"/>
+      <c r="Z3" s="8"/>
+      <c r="AA3" s="9"/>
+      <c r="AB3" s="8"/>
+      <c r="AC3" s="9"/>
+      <c r="AD3" s="8"/>
+      <c r="AE3" s="8"/>
+      <c r="AF3" s="8"/>
+      <c r="AG3" s="8"/>
+    </row>
+    <row r="4" spans="1:34" s="14" customFormat="1" ht="108" x14ac:dyDescent="0.2">
+      <c r="A4" s="13"/>
+      <c r="B4" s="7">
+        <f>3+1</f>
+        <v>4</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="L4" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="M4" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="N4" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="O4" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="P4" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q4" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="R4" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="S4" s="10"/>
+      <c r="T4" s="10"/>
+      <c r="U4" s="10"/>
+      <c r="V4" s="10"/>
+      <c r="W4" s="10"/>
+      <c r="X4" s="10"/>
+      <c r="Y4" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z4" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA4" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB4" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC4" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="AA3" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="AB3" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="AC3" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="AD3" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="AE3" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="AF3" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="AG3" s="8" t="s">
+      <c r="AD4" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="AE4" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="AF4" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="AG4" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="AH3" s="3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="4" spans="1:34" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="15"/>
-      <c r="B4" s="16">
-        <f t="shared" ref="B4:B8" si="0">B3+1</f>
-        <v>5</v>
-      </c>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
-      <c r="O4" s="9"/>
-      <c r="P4" s="9"/>
-      <c r="Q4" s="9"/>
-      <c r="R4" s="9"/>
-      <c r="S4" s="17"/>
-      <c r="T4" s="17"/>
-      <c r="U4" s="17"/>
-      <c r="V4" s="17"/>
-      <c r="W4" s="17"/>
-      <c r="X4" s="17"/>
-      <c r="Y4" s="9"/>
-      <c r="Z4" s="9"/>
-      <c r="AA4" s="9"/>
-      <c r="AB4" s="9"/>
-      <c r="AC4" s="9"/>
-      <c r="AD4" s="8"/>
-      <c r="AE4" s="8"/>
-      <c r="AF4" s="8"/>
-      <c r="AG4" s="9"/>
+      <c r="AH4" s="3" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="5" spans="1:34" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6"/>
       <c r="B5" s="8">
-        <f t="shared" si="0"/>
-        <v>6</v>
+        <f t="shared" ref="B4:B8" si="0">B4+1</f>
+        <v>5</v>
       </c>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -1537,11 +1510,11 @@
       <c r="AF5" s="8"/>
       <c r="AG5" s="8"/>
     </row>
-    <row r="6" spans="1:34" s="20" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="21"/>
+    <row r="6" spans="1:34" s="16" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="17"/>
       <c r="B6" s="9">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>
@@ -1580,7 +1553,7 @@
       <c r="A7" s="6"/>
       <c r="B7" s="7">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
@@ -1618,7 +1591,7 @@
       <c r="A8" s="6"/>
       <c r="B8" s="7">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
@@ -1654,12 +1627,12 @@
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.2">
       <c r="L9" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="Q3" r:id="rId1" xr:uid="{33C88A91-911C-4ACE-A851-B469285335A7}"/>
+    <hyperlink ref="Q4" r:id="rId1" xr:uid="{C2C9D917-AA6F-4DC4-8D1A-9D1ED78AC698}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>